<commit_message>
Auto commit on save
</commit_message>
<xml_diff>
--- a/config/argumet_loans.xlsx
+++ b/config/argumet_loans.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\python\ind_prepro\source\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\task_folder\sources\IND_prep\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="4425" yWindow="1065" windowWidth="20550" windowHeight="11385"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="17715" windowHeight="5865"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>y_col</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -156,6 +156,28 @@
   </si>
   <si>
     <t>dict_col</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>vector_to_pca_cols</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>base_to_decimal_cols</t>
+  </si>
+  <si>
+    <t>sentence_embed_cols</t>
+  </si>
+  <si>
+    <t>vector1, vector2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>non_dec1, non_dec2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>sentence1, sentence2</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -205,7 +227,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -220,6 +242,9 @@
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -535,7 +560,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="25.25" style="1" customWidth="1"/>
@@ -684,6 +709,30 @@
         <v>29</v>
       </c>
     </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B20" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>32</v>
+      </c>
+      <c r="B21" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>33</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>